<commit_message>
intraday changed behavior multi runs
intraday changed behavior multi runs
</commit_message>
<xml_diff>
--- a/ibkr-gerchik-bot/memory/reports/premarket_levels_20260430.xlsx
+++ b/ibkr-gerchik-bot/memory/reports/premarket_levels_20260430.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,37 +476,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>02/12/26</t>
+          <t>02/11/26</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>02/04/26</t>
+          <t>02/06/26</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>275.72</v>
+        <v>280.18</v>
       </c>
       <c r="E2" t="n">
-        <v>275.2</v>
+        <v>279.63</v>
       </c>
       <c r="F2" t="n">
-        <v>276.63</v>
+        <v>281.46</v>
       </c>
       <c r="G2" t="n">
-        <v>31</v>
+        <v>3</v>
       </c>
       <c r="H2" t="n">
-        <v>51.83</v>
+        <v>5.17</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>abnormal_candle</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>abnormal_candle, consolidation, historical, structural</t>
+          <t>historical, structural</t>
         </is>
       </c>
     </row>
@@ -518,7 +518,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>04/20/26</t>
+          <t>04/30/26</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -527,28 +527,28 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>274.28</v>
+        <v>276</v>
       </c>
       <c r="E3" t="n">
-        <v>273.76</v>
+        <v>275.17</v>
       </c>
       <c r="F3" t="n">
-        <v>274.8</v>
+        <v>276.66</v>
       </c>
       <c r="G3" t="n">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="H3" t="n">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>consolidation</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>historical, structural</t>
+          <t>abnormal_candle, consolidation, historical, structural</t>
         </is>
       </c>
     </row>
@@ -572,16 +572,16 @@
         <v>273.2</v>
       </c>
       <c r="E4" t="n">
-        <v>272.68</v>
+        <v>272.65</v>
       </c>
       <c r="F4" t="n">
-        <v>273.72</v>
+        <v>274.83</v>
       </c>
       <c r="G4" t="n">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="H4" t="n">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -614,16 +614,16 @@
         <v>270.71</v>
       </c>
       <c r="E5" t="n">
-        <v>270.19</v>
+        <v>270.16</v>
       </c>
       <c r="F5" t="n">
-        <v>271.58</v>
+        <v>271.61</v>
       </c>
       <c r="G5" t="n">
         <v>26</v>
       </c>
       <c r="H5" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -656,16 +656,16 @@
         <v>262.19</v>
       </c>
       <c r="E6" t="n">
-        <v>261.64</v>
+        <v>261.61</v>
       </c>
       <c r="F6" t="n">
-        <v>263</v>
+        <v>263.03</v>
       </c>
       <c r="G6" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H6" t="n">
-        <v>61.66</v>
+        <v>62.66</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -698,10 +698,10 @@
         <v>260.18</v>
       </c>
       <c r="E7" t="n">
-        <v>259.61</v>
+        <v>259.58</v>
       </c>
       <c r="F7" t="n">
-        <v>260.7</v>
+        <v>260.73</v>
       </c>
       <c r="G7" t="n">
         <v>36</v>
@@ -740,10 +740,10 @@
         <v>258.86</v>
       </c>
       <c r="E8" t="n">
-        <v>257.64</v>
+        <v>257.61</v>
       </c>
       <c r="F8" t="n">
-        <v>259.38</v>
+        <v>259.41</v>
       </c>
       <c r="G8" t="n">
         <v>43</v>
@@ -782,16 +782,16 @@
         <v>253.98</v>
       </c>
       <c r="E9" t="n">
-        <v>252.98</v>
+        <v>252.95</v>
       </c>
       <c r="F9" t="n">
-        <v>254.5</v>
+        <v>254.53</v>
       </c>
       <c r="G9" t="n">
         <v>45</v>
       </c>
       <c r="H9" t="n">
-        <v>62.42</v>
+        <v>64.42</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -824,16 +824,16 @@
         <v>250.65</v>
       </c>
       <c r="E10" t="n">
-        <v>250.13</v>
+        <v>248.97</v>
       </c>
       <c r="F10" t="n">
-        <v>251.17</v>
+        <v>251.2</v>
       </c>
       <c r="G10" t="n">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="H10" t="n">
-        <v>15.42</v>
+        <v>41.42</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -854,37 +854,37 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>03/24/26</t>
+          <t>03/23/26</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>03/13/26</t>
+          <t>03/19/26</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>249.55</v>
+        <v>247.99</v>
       </c>
       <c r="E11" t="n">
-        <v>249</v>
+        <v>247.44</v>
       </c>
       <c r="F11" t="n">
-        <v>250.07</v>
+        <v>248.54</v>
       </c>
       <c r="G11" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="H11" t="n">
-        <v>27.42</v>
+        <v>11.42</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>gap</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>historical, structural</t>
+          <t>gap</t>
         </is>
       </c>
     </row>
@@ -896,70 +896,70 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>03/23/26</t>
+          <t>03/20/26</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>03/19/26</t>
+          <t>03/20/26</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>247.99</v>
+        <v>246</v>
       </c>
       <c r="E12" t="n">
-        <v>247.47</v>
+        <v>244.96</v>
       </c>
       <c r="F12" t="n">
-        <v>248.51</v>
+        <v>246.55</v>
       </c>
       <c r="G12" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H12" t="n">
-        <v>11.42</v>
+        <v>15.42</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>gap</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>gap</t>
+          <t>consolidation, historical, structural</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>03/20/26</t>
+          <t>04/24/26</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>03/20/26</t>
+          <t>04/24/26</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>246</v>
+        <v>264.5</v>
       </c>
       <c r="E13" t="n">
-        <v>244.99</v>
+        <v>263.8</v>
       </c>
       <c r="F13" t="n">
-        <v>246.52</v>
+        <v>265.2</v>
       </c>
       <c r="G13" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H13" t="n">
-        <v>15.42</v>
+        <v>12.75</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -968,7 +968,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>consolidation, historical, structural</t>
+          <t>historical, structural</t>
         </is>
       </c>
     </row>
@@ -980,37 +980,37 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>04/30/26</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>04/24/26</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>04/24/26</t>
-        </is>
-      </c>
       <c r="D14" t="n">
-        <v>264.5</v>
+        <v>263.04</v>
       </c>
       <c r="E14" t="n">
-        <v>263.8</v>
+        <v>262.34</v>
       </c>
       <c r="F14" t="n">
-        <v>265.2</v>
+        <v>263.74</v>
       </c>
       <c r="G14" t="n">
         <v>4</v>
       </c>
       <c r="H14" t="n">
-        <v>10.75</v>
+        <v>10</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>gap</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>historical, structural</t>
+          <t>gap</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>04/30/26</t>
+          <t>04/28/26</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1031,19 +1031,19 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>263.04</v>
+        <v>261.12</v>
       </c>
       <c r="E15" t="n">
-        <v>262.34</v>
+        <v>259.28</v>
       </c>
       <c r="F15" t="n">
-        <v>263.74</v>
+        <v>261.82</v>
       </c>
       <c r="G15" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H15" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1069,23 +1069,23 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>04/24/26</t>
+          <t>04/23/26</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>261.12</v>
+        <v>258.39</v>
       </c>
       <c r="E16" t="n">
-        <v>259.28</v>
+        <v>257.69</v>
       </c>
       <c r="F16" t="n">
-        <v>261.82</v>
+        <v>259.09</v>
       </c>
       <c r="G16" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H16" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1106,28 +1106,28 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>04/28/26</t>
+          <t>04/21/26</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>04/23/26</t>
+          <t>04/17/26</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>258.39</v>
+        <v>255.09</v>
       </c>
       <c r="E17" t="n">
-        <v>257.69</v>
+        <v>254.16</v>
       </c>
       <c r="F17" t="n">
-        <v>259.09</v>
+        <v>255.79</v>
       </c>
       <c r="G17" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="H17" t="n">
-        <v>9</v>
+        <v>27.83</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1148,28 +1148,28 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>04/21/26</t>
+          <t>04/22/26</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>04/17/26</t>
+          <t>04/14/26</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>255.09</v>
+        <v>252.54</v>
       </c>
       <c r="E18" t="n">
-        <v>254.16</v>
+        <v>251.48</v>
       </c>
       <c r="F18" t="n">
-        <v>255.79</v>
+        <v>253.24</v>
       </c>
       <c r="G18" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="H18" t="n">
-        <v>27.83</v>
+        <v>12.83</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>gap</t>
+          <t>gap, historical, structural</t>
         </is>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>04/22/26</t>
+          <t>04/20/26</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1199,28 +1199,28 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>252.54</v>
+        <v>245.36</v>
       </c>
       <c r="E19" t="n">
-        <v>251.48</v>
+        <v>243.5</v>
       </c>
       <c r="F19" t="n">
-        <v>253.24</v>
+        <v>246.06</v>
       </c>
       <c r="G19" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H19" t="n">
-        <v>12.83</v>
+        <v>8.73</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>gap</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>gap, historical, structural</t>
+          <t>historical, structural</t>
         </is>
       </c>
     </row>
@@ -1232,28 +1232,28 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>04/20/26</t>
+          <t>04/10/26</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>04/14/26</t>
+          <t>04/10/26</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>245.36</v>
+        <v>240.43</v>
       </c>
       <c r="E20" t="n">
-        <v>243.5</v>
+        <v>239.73</v>
       </c>
       <c r="F20" t="n">
-        <v>246.06</v>
+        <v>241.13</v>
       </c>
       <c r="G20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H20" t="n">
-        <v>8.73</v>
+        <v>7.56</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1274,37 +1274,37 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>04/10/26</t>
+          <t>02/05/26</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>04/10/26</t>
+          <t>02/04/26</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>240.43</v>
+        <v>232.99</v>
       </c>
       <c r="E21" t="n">
-        <v>239.73</v>
+        <v>232.29</v>
       </c>
       <c r="F21" t="n">
-        <v>241.13</v>
+        <v>233.69</v>
       </c>
       <c r="G21" t="n">
         <v>2</v>
       </c>
       <c r="H21" t="n">
-        <v>7.56</v>
+        <v>9.49</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>gap</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>historical, structural</t>
+          <t>gap</t>
         </is>
       </c>
     </row>
@@ -1316,37 +1316,37 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>03/05/26</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
           <t>02/05/26</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>02/04/26</t>
-        </is>
-      </c>
       <c r="D22" t="n">
-        <v>232.99</v>
+        <v>220.47</v>
       </c>
       <c r="E22" t="n">
-        <v>232.29</v>
+        <v>219.77</v>
       </c>
       <c r="F22" t="n">
-        <v>233.69</v>
+        <v>221.17</v>
       </c>
       <c r="G22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H22" t="n">
-        <v>9.49</v>
+        <v>6.46</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>gap</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>gap</t>
+          <t>historical, structural</t>
         </is>
       </c>
     </row>
@@ -1563,33 +1563,33 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>BBBY</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>02/10/26</t>
+          <t>04/20/26</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>02/10/26</t>
+          <t>04/20/26</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>423.68</v>
+        <v>6.27</v>
       </c>
       <c r="E28" t="n">
-        <v>422.48</v>
+        <v>6.21</v>
       </c>
       <c r="F28" t="n">
-        <v>426.02</v>
+        <v>6.33</v>
       </c>
       <c r="G28" t="n">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="H28" t="n">
-        <v>76.97</v>
+        <v>6.93</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>gap, historical, structural</t>
+          <t>historical, structural</t>
         </is>
       </c>
     </row>
@@ -1610,37 +1610,37 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>04/17/26</t>
+          <t>02/10/26</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>02/04/26</t>
+          <t>02/10/26</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>420.26</v>
+        <v>423.68</v>
       </c>
       <c r="E29" t="n">
-        <v>418.41</v>
+        <v>422.48</v>
       </c>
       <c r="F29" t="n">
-        <v>421.46</v>
+        <v>426.02</v>
       </c>
       <c r="G29" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H29" t="n">
-        <v>51.97</v>
+        <v>76.97</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>gap</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>gap</t>
+          <t>gap, historical, structural</t>
         </is>
       </c>
     </row>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>04/20/26</t>
+          <t>04/17/26</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1661,28 +1661,28 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>416.3</v>
+        <v>420.26</v>
       </c>
       <c r="E30" t="n">
-        <v>415.1</v>
+        <v>418.41</v>
       </c>
       <c r="F30" t="n">
-        <v>417.5</v>
+        <v>421.46</v>
       </c>
       <c r="G30" t="n">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="H30" t="n">
-        <v>14.9</v>
+        <v>51.97</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>gap</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>historical, structural</t>
+          <t>gap</t>
         </is>
       </c>
     </row>
@@ -1694,37 +1694,37 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>02/05/26</t>
+          <t>04/20/26</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>02/05/26</t>
+          <t>02/04/26</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>408</v>
+        <v>416.3</v>
       </c>
       <c r="E31" t="n">
-        <v>406.29</v>
+        <v>415.1</v>
       </c>
       <c r="F31" t="n">
-        <v>409.2</v>
+        <v>417.5</v>
       </c>
       <c r="G31" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="H31" t="n">
-        <v>35</v>
+        <v>14.9</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>gap</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>gap, historical, structural</t>
+          <t>historical, structural</t>
         </is>
       </c>
     </row>
@@ -1736,7 +1736,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>02/26/26</t>
+          <t>02/05/26</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1745,19 +1745,19 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>404.71</v>
+        <v>408</v>
       </c>
       <c r="E32" t="n">
-        <v>403.2</v>
+        <v>406.29</v>
       </c>
       <c r="F32" t="n">
-        <v>405.91</v>
+        <v>409.2</v>
       </c>
       <c r="G32" t="n">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="H32" t="n">
-        <v>84</v>
+        <v>35</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -1778,32 +1778,32 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>04/08/26</t>
+          <t>02/26/26</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>02/23/26</t>
+          <t>02/05/26</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>385</v>
+        <v>404.71</v>
       </c>
       <c r="E33" t="n">
-        <v>383.78</v>
+        <v>403.2</v>
       </c>
       <c r="F33" t="n">
-        <v>388.41</v>
+        <v>405.91</v>
       </c>
       <c r="G33" t="n">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="H33" t="n">
-        <v>29.59</v>
+        <v>84</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>gap</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -1820,28 +1820,28 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>02/24/26</t>
+          <t>04/08/26</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>02/24/26</t>
+          <t>02/23/26</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>381.71</v>
+        <v>385</v>
       </c>
       <c r="E34" t="n">
-        <v>378.92</v>
+        <v>383.78</v>
       </c>
       <c r="F34" t="n">
-        <v>382.91</v>
+        <v>388.41</v>
       </c>
       <c r="G34" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="H34" t="n">
-        <v>15.56</v>
+        <v>29.59</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>historical, structural</t>
+          <t>gap, historical, structural</t>
         </is>
       </c>
     </row>
@@ -1862,37 +1862,37 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>03/25/26</t>
+          <t>02/24/26</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>03/24/26</t>
+          <t>02/24/26</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>376.93</v>
+        <v>381.71</v>
       </c>
       <c r="E35" t="n">
-        <v>375.73</v>
+        <v>378.92</v>
       </c>
       <c r="F35" t="n">
-        <v>378.13</v>
+        <v>382.91</v>
       </c>
       <c r="G35" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H35" t="n">
-        <v>7.56</v>
+        <v>15.56</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>gap</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>gap</t>
+          <t>historical, structural</t>
         </is>
       </c>
     </row>
@@ -1913,19 +1913,19 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>372.74</v>
+        <v>376.93</v>
       </c>
       <c r="E36" t="n">
-        <v>371.09</v>
+        <v>375.73</v>
       </c>
       <c r="F36" t="n">
-        <v>373.94</v>
+        <v>378.13</v>
       </c>
       <c r="G36" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="H36" t="n">
-        <v>47.56</v>
+        <v>7.56</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -1941,75 +1941,75 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SANM</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>04/28/26</t>
+          <t>03/25/26</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>04/28/26</t>
+          <t>03/24/26</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>230.56</v>
+        <v>372.74</v>
       </c>
       <c r="E37" t="n">
-        <v>228.55</v>
+        <v>371.09</v>
       </c>
       <c r="F37" t="n">
-        <v>232.57</v>
+        <v>373.94</v>
       </c>
       <c r="G37" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="H37" t="n">
-        <v>7.93</v>
+        <v>47.56</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>abnormal_candle</t>
+          <t>gap</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>abnormal_candle, consolidation, historical, structural</t>
+          <t>gap</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SANM</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>04/29/26</t>
+          <t>03/27/26</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>04/28/26</t>
+          <t>03/27/26</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>215.46</v>
+        <v>361.9</v>
       </c>
       <c r="E38" t="n">
-        <v>211.78</v>
+        <v>360.7</v>
       </c>
       <c r="F38" t="n">
-        <v>219.68</v>
+        <v>363.1</v>
       </c>
       <c r="G38" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H38" t="n">
-        <v>21</v>
+        <v>6.29</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>04/30/26</t>
+          <t>04/28/26</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2039,28 +2039,28 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>208.67</v>
+        <v>230.56</v>
       </c>
       <c r="E39" t="n">
-        <v>202.97</v>
+        <v>228.55</v>
       </c>
       <c r="F39" t="n">
-        <v>210.68</v>
+        <v>232.57</v>
       </c>
       <c r="G39" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H39" t="n">
-        <v>12</v>
+        <v>7.93</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>gap</t>
+          <t>abnormal_candle</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>gap</t>
+          <t>abnormal_candle, consolidation, historical, structural</t>
         </is>
       </c>
     </row>
@@ -2072,196 +2072,196 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>04/16/26</t>
+          <t>04/29/26</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>04/16/26</t>
+          <t>04/28/26</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>172.35</v>
+        <v>217.67</v>
       </c>
       <c r="E40" t="n">
-        <v>166.96</v>
+        <v>211.78</v>
       </c>
       <c r="F40" t="n">
-        <v>174.36</v>
+        <v>219.68</v>
       </c>
       <c r="G40" t="n">
+        <v>9</v>
+      </c>
+      <c r="H40" t="n">
         <v>19</v>
       </c>
-      <c r="H40" t="n">
-        <v>33.83</v>
-      </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>abnormal_candle</t>
+          <t>gap</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>abnormal_candle, gap, historical, structural</t>
+          <t>gap</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SEI</t>
+          <t>SANM</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>04/30/26</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
           <t>04/28/26</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>04/28/26</t>
-        </is>
-      </c>
       <c r="D41" t="n">
-        <v>81.23999999999999</v>
+        <v>208.67</v>
       </c>
       <c r="E41" t="n">
-        <v>79.89</v>
+        <v>202.97</v>
       </c>
       <c r="F41" t="n">
-        <v>82.12</v>
+        <v>210.68</v>
       </c>
       <c r="G41" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H41" t="n">
-        <v>12.97</v>
+        <v>12</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>abnormal_candle</t>
+          <t>gap</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>abnormal_candle, consolidation, historical, structural</t>
+          <t>gap</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SEI</t>
+          <t>SANM</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>04/29/26</t>
+          <t>04/16/26</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>04/24/26</t>
+          <t>04/16/26</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>74.44</v>
+        <v>172.35</v>
       </c>
       <c r="E42" t="n">
-        <v>73.56</v>
+        <v>166.96</v>
       </c>
       <c r="F42" t="n">
-        <v>75.31999999999999</v>
+        <v>174.36</v>
       </c>
       <c r="G42" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="H42" t="n">
-        <v>13</v>
+        <v>33.83</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>gap</t>
+          <t>abnormal_candle</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>gap</t>
+          <t>abnormal_candle, gap, historical, structural</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>SEI</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>03/11/26</t>
+          <t>04/28/26</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>02/04/26</t>
+          <t>04/28/26</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>416.38</v>
+        <v>81.23999999999999</v>
       </c>
       <c r="E43" t="n">
-        <v>414.9</v>
+        <v>79.89</v>
       </c>
       <c r="F43" t="n">
-        <v>418.92</v>
+        <v>82.12</v>
       </c>
       <c r="G43" t="n">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="H43" t="n">
-        <v>54.81</v>
+        <v>12.97</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>abnormal_candle</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>gap, historical, structural</t>
+          <t>abnormal_candle, consolidation, historical, structural</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>SEI</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>02/23/26</t>
+          <t>04/28/26</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>02/04/26</t>
+          <t>04/28/26</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>411.82</v>
+        <v>77.12</v>
       </c>
       <c r="E44" t="n">
-        <v>410.34</v>
+        <v>76.23999999999999</v>
       </c>
       <c r="F44" t="n">
-        <v>413.84</v>
+        <v>78</v>
       </c>
       <c r="G44" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="H44" t="n">
-        <v>43.81</v>
+        <v>7</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
@@ -2277,33 +2277,33 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>SEI</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>04/08/26</t>
+          <t>04/29/26</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>04/06/26</t>
+          <t>04/24/26</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>346.65</v>
+        <v>74.44</v>
       </c>
       <c r="E45" t="n">
-        <v>344.79</v>
+        <v>73.56</v>
       </c>
       <c r="F45" t="n">
-        <v>348.13</v>
+        <v>75.31999999999999</v>
       </c>
       <c r="G45" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H45" t="n">
-        <v>21.53</v>
+        <v>13</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -2324,35 +2324,203 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
+          <t>02/11/26</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>02/11/26</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>436.35</v>
+      </c>
+      <c r="E46" t="n">
+        <v>434.87</v>
+      </c>
+      <c r="F46" t="n">
+        <v>437.83</v>
+      </c>
+      <c r="G46" t="n">
+        <v>2</v>
+      </c>
+      <c r="H46" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>historical</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>historical, structural</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>03/11/26</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>02/04/26</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>416.38</v>
+      </c>
+      <c r="E47" t="n">
+        <v>414.9</v>
+      </c>
+      <c r="F47" t="n">
+        <v>418.92</v>
+      </c>
+      <c r="G47" t="n">
+        <v>28</v>
+      </c>
+      <c r="H47" t="n">
+        <v>54.81</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>historical</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>gap, historical, structural</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>02/23/26</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>02/04/26</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>411.82</v>
+      </c>
+      <c r="E48" t="n">
+        <v>410.34</v>
+      </c>
+      <c r="F48" t="n">
+        <v>413.84</v>
+      </c>
+      <c r="G48" t="n">
+        <v>23</v>
+      </c>
+      <c r="H48" t="n">
+        <v>43.81</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>gap</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>04/08/26</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>04/06/26</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>346.65</v>
+      </c>
+      <c r="E49" t="n">
+        <v>344.79</v>
+      </c>
+      <c r="F49" t="n">
+        <v>348.13</v>
+      </c>
+      <c r="G49" t="n">
+        <v>10</v>
+      </c>
+      <c r="H49" t="n">
+        <v>21.53</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>gap</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
           <t>04/09/26</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>04/07/26</t>
         </is>
       </c>
-      <c r="D46" t="n">
+      <c r="D50" t="n">
         <v>337.25</v>
       </c>
-      <c r="E46" t="n">
+      <c r="E50" t="n">
         <v>335.76</v>
       </c>
-      <c r="F46" t="n">
+      <c r="F50" t="n">
         <v>338.73</v>
       </c>
-      <c r="G46" t="n">
+      <c r="G50" t="n">
         <v>6</v>
       </c>
-      <c r="H46" t="n">
+      <c r="H50" t="n">
         <v>9.49</v>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="I50" t="inlineStr">
         <is>
           <t>historical</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="J50" t="inlineStr">
         <is>
           <t>consolidation, historical, structural</t>
         </is>

</xml_diff>